<commit_message>
updated the week3 lecture 2
</commit_message>
<xml_diff>
--- a/Week03/what-if-analysis.xlsx
+++ b/Week03/what-if-analysis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dhruv\Downloads\BA-L\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dhruv\Downloads\BA-L\Week03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{428616C1-EE54-4EF7-921B-3C5EF06CC400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38C4084-5568-4C5D-BA6D-907E176DA9E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{3F1BB861-918F-4285-983B-99B972B04A7E}"/>
   </bookViews>
@@ -350,26 +350,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -384,15 +377,21 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -741,170 +740,169 @@
   <sheetData>
     <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
     </row>
     <row r="3" spans="2:7" ht="15.6" collapsed="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="14" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="21.6" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="16" t="s">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="E4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="13" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
     </row>
     <row r="6" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="10"/>
-      <c r="C6" s="10" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6">
         <v>1300</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="12">
         <v>1200</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="12">
         <v>1100</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="12">
         <v>1300</v>
       </c>
     </row>
     <row r="7" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="10"/>
-      <c r="C7" s="10" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7">
         <v>6500</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="12">
         <v>5000</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="12">
         <v>3500</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="12">
         <v>6500</v>
       </c>
     </row>
     <row r="8" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="10"/>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8">
         <v>650</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="12">
         <v>700</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="12">
         <v>750</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="12">
         <v>650</v>
       </c>
     </row>
     <row r="9" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="10"/>
-      <c r="C9" s="10" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9">
         <v>700000</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="12">
         <v>500000</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="12">
         <v>400000</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="12">
         <v>700000</v>
       </c>
     </row>
     <row r="10" spans="2:7" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="10"/>
-      <c r="C10" s="10" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10">
         <v>800000</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="12">
         <v>800000</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="12">
         <v>800000</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="12">
         <v>800000</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
     </row>
     <row r="12" spans="2:7" ht="15" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="12"/>
-      <c r="C12" s="12" t="s">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>0.32248520710059198</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="3">
         <v>0.2</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="3">
         <v>6.4935064935064896E-3</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="3">
         <v>0.32248520710059198</v>
       </c>
     </row>
@@ -938,38 +936,38 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="18"/>
+      <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B4">
         <v>1300</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E4">
@@ -983,13 +981,13 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B5">
         <v>6500</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E5">
@@ -1003,13 +1001,13 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B6">
         <v>650</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E6">
@@ -1023,13 +1021,13 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B7">
         <v>700000</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="E7">
@@ -1043,13 +1041,13 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B8">
         <v>800000</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="E8">
@@ -1063,7 +1061,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B10">
@@ -1072,7 +1070,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B11">
@@ -1081,7 +1079,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B12">
@@ -1090,7 +1088,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B13">
@@ -1194,19 +1192,19 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="D2" s="17" t="s">
+      <c r="B2" s="15"/>
+      <c r="D2" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1289,57 +1287,57 @@
         <f>(B3-B5)*B4 - B6</f>
         <v>120000</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="17"/>
+      <c r="B11" s="15"/>
       <c r="D11">
         <f>B8</f>
         <v>120000</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="14">
         <v>500</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="14">
         <v>1000</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="14">
         <v>1500</v>
       </c>
-      <c r="H11" s="18">
+      <c r="H11" s="14">
         <v>2000</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="14">
         <v>2500</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="14">
         <v>3000</v>
       </c>
-      <c r="K11" s="18">
+      <c r="K11" s="14">
         <v>3500</v>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="14">
         <v>4000</v>
       </c>
-      <c r="M11" s="18">
+      <c r="M11" s="14">
         <v>4500</v>
       </c>
     </row>
@@ -1351,7 +1349,7 @@
         <f>B8</f>
         <v>120000</v>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="14">
         <v>300</v>
       </c>
       <c r="E12">
@@ -1391,7 +1389,7 @@
         <f t="dataTable" ref="B13:B20" dt2D="0" dtr="0" r1="B3"/>
         <v>20000</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="14">
         <v>400</v>
       </c>
       <c r="E13">
@@ -1429,7 +1427,7 @@
       <c r="B14">
         <v>70000</v>
       </c>
-      <c r="D14" s="18">
+      <c r="D14" s="14">
         <v>500</v>
       </c>
       <c r="E14">
@@ -1467,10 +1465,10 @@
       <c r="B15">
         <v>120000</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="14">
         <v>600</v>
       </c>
       <c r="E15">
@@ -1508,8 +1506,8 @@
       <c r="B16">
         <v>170000</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="18">
+      <c r="C16" s="16"/>
+      <c r="D16" s="14">
         <v>700</v>
       </c>
       <c r="E16">
@@ -1547,8 +1545,8 @@
       <c r="B17">
         <v>220000</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="18">
+      <c r="C17" s="16"/>
+      <c r="D17" s="14">
         <v>800</v>
       </c>
       <c r="E17">
@@ -1586,8 +1584,8 @@
       <c r="B18">
         <v>270000</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="18">
+      <c r="C18" s="16"/>
+      <c r="D18" s="14">
         <v>900</v>
       </c>
       <c r="E18">
@@ -1625,7 +1623,7 @@
       <c r="B19">
         <v>320000</v>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="14">
         <v>1000</v>
       </c>
       <c r="E19">
@@ -1663,7 +1661,7 @@
       <c r="B20">
         <v>370000</v>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="14">
         <v>1100</v>
       </c>
       <c r="E20">
@@ -1695,7 +1693,7 @@
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D21" s="18">
+      <c r="D21" s="14">
         <v>1200</v>
       </c>
       <c r="E21">
@@ -1727,7 +1725,7 @@
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D22" s="18">
+      <c r="D22" s="14">
         <v>1300</v>
       </c>
       <c r="E22">
@@ -1759,7 +1757,7 @@
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D23" s="18">
+      <c r="D23" s="14">
         <v>1400</v>
       </c>
       <c r="E23">

</xml_diff>